<commit_message>
Change export excel template version, drop old templates
</commit_message>
<xml_diff>
--- a/ckanext/lhm/schemas/template_gdp.xlsx
+++ b/ckanext/lhm/schemas/template_gdp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\home\mb\p2\ckanext-lhm\ckanext\lhm\schemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D20CC6D9-9435-42C2-9AED-E9C15220DD4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56CFA98F-4F2C-4599-A9B5-D578F5D03B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="21792" windowHeight="11772" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadaten" sheetId="1" r:id="rId1"/>
@@ -770,7 +770,7 @@
     <t>Bedeutung</t>
   </si>
   <si>
-    <t>1.2.5.</t>
+    <t>1.3.1.</t>
   </si>
 </sst>
 </file>
@@ -1037,14 +1037,14 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1810,7 +1810,7 @@
       <c r="K27" s="19"/>
     </row>
     <row r="28" spans="1:12">
-      <c r="A28" s="31" t="s">
+      <c r="A28" s="29" t="s">
         <v>105</v>
       </c>
       <c r="B28" s="19"/>
@@ -1901,60 +1901,60 @@
       </c>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" s="29" t="s">
+      <c r="A37" s="30" t="s">
         <v>195</v>
       </c>
-      <c r="B37" s="30"/>
-      <c r="C37" s="30"/>
-      <c r="D37" s="30"/>
+      <c r="B37" s="31"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="30"/>
-      <c r="B38" s="30"/>
-      <c r="C38" s="30"/>
-      <c r="D38" s="30"/>
+      <c r="A38" s="31"/>
+      <c r="B38" s="31"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="31"/>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" s="30"/>
-      <c r="B39" s="30"/>
-      <c r="C39" s="30"/>
-      <c r="D39" s="30"/>
+      <c r="A39" s="31"/>
+      <c r="B39" s="31"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="31"/>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" s="30"/>
-      <c r="B40" s="30"/>
-      <c r="C40" s="30"/>
-      <c r="D40" s="30"/>
+      <c r="A40" s="31"/>
+      <c r="B40" s="31"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
     </row>
     <row r="41" spans="1:4">
-      <c r="A41" s="30"/>
-      <c r="B41" s="30"/>
-      <c r="C41" s="30"/>
-      <c r="D41" s="30"/>
+      <c r="A41" s="31"/>
+      <c r="B41" s="31"/>
+      <c r="C41" s="31"/>
+      <c r="D41" s="31"/>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="30"/>
-      <c r="B42" s="30"/>
-      <c r="C42" s="30"/>
-      <c r="D42" s="30"/>
+      <c r="A42" s="31"/>
+      <c r="B42" s="31"/>
+      <c r="C42" s="31"/>
+      <c r="D42" s="31"/>
     </row>
     <row r="43" spans="1:4">
-      <c r="A43" s="30"/>
-      <c r="B43" s="30"/>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
+      <c r="A43" s="31"/>
+      <c r="B43" s="31"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="31"/>
     </row>
     <row r="44" spans="1:4">
-      <c r="A44" s="30"/>
-      <c r="B44" s="30"/>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
+      <c r="A44" s="31"/>
+      <c r="B44" s="31"/>
+      <c r="C44" s="31"/>
+      <c r="D44" s="31"/>
     </row>
     <row r="45" spans="1:4">
-      <c r="A45" s="30"/>
-      <c r="B45" s="30"/>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
+      <c r="A45" s="31"/>
+      <c r="B45" s="31"/>
+      <c r="C45" s="31"/>
+      <c r="D45" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Make private datasets exportable: Change from api calls to internal actions, change export excel template version, drop old templates
</commit_message>
<xml_diff>
--- a/ckanext/lhm/schemas/template_gdp.xlsx
+++ b/ckanext/lhm/schemas/template_gdp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\home\mb\p2\ckanext-lhm\ckanext\lhm\schemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D20CC6D9-9435-42C2-9AED-E9C15220DD4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABEC6B3D-26B2-479D-871F-39372DD47D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="21792" windowHeight="11772" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadaten" sheetId="1" r:id="rId1"/>
@@ -770,7 +770,7 @@
     <t>Bedeutung</t>
   </si>
   <si>
-    <t>1.2.5.</t>
+    <t>1.3.1.</t>
   </si>
 </sst>
 </file>
@@ -1037,14 +1037,14 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1810,7 +1810,7 @@
       <c r="K27" s="19"/>
     </row>
     <row r="28" spans="1:12">
-      <c r="A28" s="31" t="s">
+      <c r="A28" s="29" t="s">
         <v>105</v>
       </c>
       <c r="B28" s="19"/>
@@ -1901,60 +1901,60 @@
       </c>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" s="29" t="s">
+      <c r="A37" s="30" t="s">
         <v>195</v>
       </c>
-      <c r="B37" s="30"/>
-      <c r="C37" s="30"/>
-      <c r="D37" s="30"/>
+      <c r="B37" s="31"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="30"/>
-      <c r="B38" s="30"/>
-      <c r="C38" s="30"/>
-      <c r="D38" s="30"/>
+      <c r="A38" s="31"/>
+      <c r="B38" s="31"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="31"/>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" s="30"/>
-      <c r="B39" s="30"/>
-      <c r="C39" s="30"/>
-      <c r="D39" s="30"/>
+      <c r="A39" s="31"/>
+      <c r="B39" s="31"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="31"/>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" s="30"/>
-      <c r="B40" s="30"/>
-      <c r="C40" s="30"/>
-      <c r="D40" s="30"/>
+      <c r="A40" s="31"/>
+      <c r="B40" s="31"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
     </row>
     <row r="41" spans="1:4">
-      <c r="A41" s="30"/>
-      <c r="B41" s="30"/>
-      <c r="C41" s="30"/>
-      <c r="D41" s="30"/>
+      <c r="A41" s="31"/>
+      <c r="B41" s="31"/>
+      <c r="C41" s="31"/>
+      <c r="D41" s="31"/>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="30"/>
-      <c r="B42" s="30"/>
-      <c r="C42" s="30"/>
-      <c r="D42" s="30"/>
+      <c r="A42" s="31"/>
+      <c r="B42" s="31"/>
+      <c r="C42" s="31"/>
+      <c r="D42" s="31"/>
     </row>
     <row r="43" spans="1:4">
-      <c r="A43" s="30"/>
-      <c r="B43" s="30"/>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
+      <c r="A43" s="31"/>
+      <c r="B43" s="31"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="31"/>
     </row>
     <row r="44" spans="1:4">
-      <c r="A44" s="30"/>
-      <c r="B44" s="30"/>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
+      <c r="A44" s="31"/>
+      <c r="B44" s="31"/>
+      <c r="C44" s="31"/>
+      <c r="D44" s="31"/>
     </row>
     <row r="45" spans="1:4">
-      <c r="A45" s="30"/>
-      <c r="B45" s="30"/>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
+      <c r="A45" s="31"/>
+      <c r="B45" s="31"/>
+      <c r="C45" s="31"/>
+      <c r="D45" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Add ArcGIS Map and Feature Service to resource formats
</commit_message>
<xml_diff>
--- a/ckanext/lhm/schemas/template_gdp.xlsx
+++ b/ckanext/lhm/schemas/template_gdp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\home\mb\p2\ckanext-lhm\ckanext\lhm\schemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56CFA98F-4F2C-4599-A9B5-D578F5D03B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD710B2B-A97F-4EF5-95C8-2F3572EB0141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
   </bookViews>
@@ -306,9 +306,6 @@
     <t>_id</t>
   </si>
   <si>
-    <t>ArcGIS Kartenservice</t>
-  </si>
-  <si>
     <t>URL</t>
   </si>
   <si>
@@ -352,9 +349,6 @@
   </si>
   <si>
     <t>XML/GML</t>
-  </si>
-  <si>
-    <t>Link</t>
   </si>
   <si>
     <t>URL / Datei</t>
@@ -770,7 +764,13 @@
     <t>Bedeutung</t>
   </si>
   <si>
-    <t>1.3.1.</t>
+    <t>ArcGIS Feature Service</t>
+  </si>
+  <si>
+    <t>ArcGIS Map Service</t>
+  </si>
+  <si>
+    <t>1.3.2.</t>
   </si>
 </sst>
 </file>
@@ -1421,7 +1421,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="18" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="12"/>
@@ -1451,7 +1451,7 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="11" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="12"/>
@@ -1466,7 +1466,7 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="16" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B5" s="21"/>
       <c r="C5" s="23"/>
@@ -1481,7 +1481,7 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="16" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B6" s="21"/>
       <c r="C6" s="21"/>
@@ -1496,7 +1496,7 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="11" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="12"/>
@@ -1511,7 +1511,7 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="11" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="12"/>
@@ -1616,7 +1616,7 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="11" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B15" s="19"/>
       <c r="C15" s="12"/>
@@ -1646,7 +1646,7 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" s="16" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B17" s="21"/>
       <c r="C17" s="12"/>
@@ -1661,7 +1661,7 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" s="16" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B18" s="21"/>
       <c r="C18" s="12"/>
@@ -1676,7 +1676,7 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="16" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B19" s="21"/>
       <c r="C19" s="12"/>
@@ -1691,7 +1691,7 @@
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="16" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B20" s="21"/>
       <c r="C20" s="12"/>
@@ -1706,7 +1706,7 @@
     </row>
     <row r="21" spans="1:12">
       <c r="A21" s="16" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B21" s="21"/>
       <c r="C21" s="12"/>
@@ -1721,7 +1721,7 @@
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="16" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B22" s="21"/>
       <c r="C22" s="21"/>
@@ -1736,7 +1736,7 @@
     </row>
     <row r="23" spans="1:12">
       <c r="A23" s="16" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B23" s="21"/>
       <c r="C23" s="12"/>
@@ -1751,7 +1751,7 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B24" s="21"/>
       <c r="C24" s="12"/>
@@ -1766,7 +1766,7 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25" s="16" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B25" s="21"/>
       <c r="C25" s="12"/>
@@ -1781,7 +1781,7 @@
     </row>
     <row r="26" spans="1:12">
       <c r="A26" s="16" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B26" s="21"/>
       <c r="C26" s="12"/>
@@ -1796,7 +1796,7 @@
     </row>
     <row r="27" spans="1:12">
       <c r="A27" s="11" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B27" s="19"/>
       <c r="C27" s="24"/>
@@ -1811,7 +1811,7 @@
     </row>
     <row r="28" spans="1:12">
       <c r="A28" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B28" s="19"/>
       <c r="C28" s="24"/>
@@ -1826,7 +1826,7 @@
     </row>
     <row r="29" spans="1:12">
       <c r="A29" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B29" s="25"/>
       <c r="C29" s="12"/>
@@ -1858,7 +1858,7 @@
     </row>
     <row r="31" spans="1:12">
       <c r="A31" s="14" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B31" s="26"/>
       <c r="C31" s="12"/>
@@ -1874,7 +1874,7 @@
     </row>
     <row r="32" spans="1:12">
       <c r="A32" s="14" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B32" s="26" t="s">
         <v>235</v>
@@ -1902,7 +1902,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="30" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B37" s="31"/>
       <c r="C37" s="31"/>
@@ -2017,10 +2017,10 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="27" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C1" s="27" t="s">
         <v>82</v>
@@ -2032,7 +2032,7 @@
         <v>81</v>
       </c>
       <c r="F1" s="27" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -2062,13 +2062,13 @@
         <v>85</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C1" s="27" t="s">
         <v>61</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -2093,16 +2093,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="27" t="s">
+        <v>186</v>
+      </c>
+      <c r="C1" s="27" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="27" t="s">
-        <v>188</v>
-      </c>
-      <c r="C1" s="27" t="s">
-        <v>89</v>
-      </c>
       <c r="D1" s="27" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -2136,7 +2136,7 @@
     <col min="15" max="15" width="14.5" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="27.3984375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="20.19921875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.796875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="22.19921875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="23.796875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="27.3984375" bestFit="1" customWidth="1"/>
@@ -2145,70 +2145,70 @@
   <sheetData>
     <row r="1" spans="1:22" s="1" customFormat="1">
       <c r="A1" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="D1" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="O1" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="Q1" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="R1" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="N1" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="R1" s="5" t="s">
+      <c r="S1" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="T1" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="U1" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="S1" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="T1" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="U1" s="5" t="s">
-        <v>222</v>
-      </c>
       <c r="V1" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" spans="1:22">
@@ -2219,60 +2219,60 @@
         <v>23</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="K2" s="3"/>
       <c r="L2" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>79</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>80</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -2283,64 +2283,64 @@
         <v>24</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="O3" s="2" t="s">
         <v>0</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -2351,31 +2351,31 @@
         <v>25</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>84</v>
@@ -2384,19 +2384,19 @@
         <v>84</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>84</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:22">
@@ -2407,34 +2407,34 @@
         <v>26</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="U5" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:22">
@@ -2445,34 +2445,34 @@
         <v>27</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="U6" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" spans="1:22">
@@ -2483,28 +2483,28 @@
         <v>28</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="N7" s="3" t="s">
         <v>17</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="U7" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" spans="1:22">
@@ -2515,28 +2515,28 @@
         <v>29</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U8" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9" spans="1:22">
@@ -2547,17 +2547,17 @@
         <v>30</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E9" s="1"/>
       <c r="G9" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>86</v>
+        <v>233</v>
       </c>
       <c r="U9" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="10" spans="1:22">
@@ -2568,18 +2568,18 @@
         <v>31</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E10" s="1"/>
       <c r="G10" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K10" s="15"/>
       <c r="R10" s="2" t="s">
-        <v>87</v>
+        <v>234</v>
       </c>
       <c r="U10" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="11" spans="1:22">
@@ -2590,18 +2590,18 @@
         <v>32</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E11" s="1"/>
       <c r="G11" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K11" s="15"/>
       <c r="R11" s="2" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="12" spans="1:22">
@@ -2612,12 +2612,12 @@
         <v>33</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E12" s="1"/>
       <c r="K12" s="15"/>
       <c r="U12" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:22">
@@ -2628,7 +2628,7 @@
         <v>34</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E13" s="1"/>
       <c r="K13" s="15"/>
@@ -2641,7 +2641,7 @@
         <v>35</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E14" s="1"/>
       <c r="K14" s="15"/>
@@ -2654,7 +2654,7 @@
         <v>36</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E15" s="1"/>
       <c r="K15" s="15"/>
@@ -2667,7 +2667,7 @@
         <v>37</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E16" s="1"/>
       <c r="K16" s="15"/>
@@ -2680,7 +2680,7 @@
         <v>38</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E17" s="1"/>
       <c r="K17" s="15"/>
@@ -2693,7 +2693,7 @@
         <v>39</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E18" s="1"/>
       <c r="K18" s="15"/>
@@ -2706,7 +2706,7 @@
         <v>40</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E19" s="1"/>
       <c r="K19" s="15"/>
@@ -2716,10 +2716,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E20" s="1"/>
       <c r="K20" s="15"/>
@@ -2732,7 +2732,7 @@
         <v>41</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E21" s="1"/>
       <c r="K21" s="15"/>
@@ -2829,7 +2829,10 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="7WMZ1mDUyvhL4UpKWt0nfcgkaCP0BpTdJaHaP4ZqioaIBj5Otagyz61Gxt0x4SOLv8AaGVTwJsZOUhjfi81XSw==" saltValue="yvb7SbXdXcRytveSJfy99Q==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="52lhtQEAIa0G0egiBOMSvDzW9IIazrxMJIqu++Msm7VrZR78YEHxwq0uV1phFxG1RVTLRGRFk7mWFXVjKblJ3g==" saltValue="LA2YV2MKD5bQ9zf69KBg+A==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V36">
+    <sortCondition sortBy="icon" ref="R9:R36"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add WMTS-KVP to resource formats
</commit_message>
<xml_diff>
--- a/ckanext/lhm/schemas/template_gdp.xlsx
+++ b/ckanext/lhm/schemas/template_gdp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\home\mb\p2\ckanext-lhm\ckanext\lhm\schemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD710B2B-A97F-4EF5-95C8-2F3572EB0141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6607627-373A-4A41-A595-EF3B4A64B030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
+    <workbookView xWindow="1056" yWindow="1452" windowWidth="21792" windowHeight="10788" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadaten" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="263">
   <si>
     <t>nein</t>
   </si>
@@ -764,13 +764,94 @@
     <t>Bedeutung</t>
   </si>
   <si>
+    <t>ArcGIS Map Service</t>
+  </si>
+  <si>
     <t>ArcGIS Feature Service</t>
   </si>
   <si>
-    <t>ArcGIS Map Service</t>
-  </si>
-  <si>
-    <t>1.3.2.</t>
+    <t>PLAN-DB</t>
+  </si>
+  <si>
+    <t>PLAN_MD_update-zyklus</t>
+  </si>
+  <si>
+    <t>Jährlich</t>
+  </si>
+  <si>
+    <t>PLAN_MD_schema</t>
+  </si>
+  <si>
+    <t>BAU</t>
+  </si>
+  <si>
+    <t>BPLAN</t>
+  </si>
+  <si>
+    <t>DENK</t>
+  </si>
+  <si>
+    <t>ENP</t>
+  </si>
+  <si>
+    <t>EWO</t>
+  </si>
+  <si>
+    <t>FIS</t>
+  </si>
+  <si>
+    <t>FNP</t>
+  </si>
+  <si>
+    <t>GEB</t>
+  </si>
+  <si>
+    <t>GEN</t>
+  </si>
+  <si>
+    <t>GRENZ</t>
+  </si>
+  <si>
+    <t>GRUEN</t>
+  </si>
+  <si>
+    <t>HAII_PRIO</t>
+  </si>
+  <si>
+    <t>INNENSTADT</t>
+  </si>
+  <si>
+    <t>LBK</t>
+  </si>
+  <si>
+    <t>REG</t>
+  </si>
+  <si>
+    <t>SIED</t>
+  </si>
+  <si>
+    <t>STAPL</t>
+  </si>
+  <si>
+    <t>UNB</t>
+  </si>
+  <si>
+    <t>ZEN</t>
+  </si>
+  <si>
+    <t>Quartalsweise</t>
+  </si>
+  <si>
+    <t>Zweijährlich</t>
+  </si>
+  <si>
+    <t>WMTS-KVP</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>1.3.3.</t>
   </si>
 </sst>
 </file>
@@ -1037,14 +1118,14 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1679,14 +1760,6 @@
         <v>150</v>
       </c>
       <c r="B19" s="21"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
       <c r="K19" s="17"/>
     </row>
     <row r="20" spans="1:12">
@@ -1694,14 +1767,6 @@
         <v>151</v>
       </c>
       <c r="B20" s="21"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
       <c r="K20" s="17"/>
     </row>
     <row r="21" spans="1:12">
@@ -1810,7 +1875,7 @@
       <c r="K27" s="19"/>
     </row>
     <row r="28" spans="1:12">
-      <c r="A28" s="29" t="s">
+      <c r="A28" s="31" t="s">
         <v>103</v>
       </c>
       <c r="B28" s="19"/>
@@ -1877,7 +1942,7 @@
         <v>202</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>235</v>
+        <v>262</v>
       </c>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
@@ -1901,60 +1966,60 @@
       </c>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" s="30" t="s">
+      <c r="A37" s="29" t="s">
         <v>193</v>
       </c>
-      <c r="B37" s="31"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="31"/>
+      <c r="B37" s="30"/>
+      <c r="C37" s="30"/>
+      <c r="D37" s="30"/>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="31"/>
-      <c r="B38" s="31"/>
-      <c r="C38" s="31"/>
-      <c r="D38" s="31"/>
+      <c r="A38" s="30"/>
+      <c r="B38" s="30"/>
+      <c r="C38" s="30"/>
+      <c r="D38" s="30"/>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" s="31"/>
-      <c r="B39" s="31"/>
-      <c r="C39" s="31"/>
-      <c r="D39" s="31"/>
+      <c r="A39" s="30"/>
+      <c r="B39" s="30"/>
+      <c r="C39" s="30"/>
+      <c r="D39" s="30"/>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" s="31"/>
-      <c r="B40" s="31"/>
-      <c r="C40" s="31"/>
-      <c r="D40" s="31"/>
+      <c r="A40" s="30"/>
+      <c r="B40" s="30"/>
+      <c r="C40" s="30"/>
+      <c r="D40" s="30"/>
     </row>
     <row r="41" spans="1:4">
-      <c r="A41" s="31"/>
-      <c r="B41" s="31"/>
-      <c r="C41" s="31"/>
-      <c r="D41" s="31"/>
+      <c r="A41" s="30"/>
+      <c r="B41" s="30"/>
+      <c r="C41" s="30"/>
+      <c r="D41" s="30"/>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="31"/>
-      <c r="B42" s="31"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="31"/>
+      <c r="A42" s="30"/>
+      <c r="B42" s="30"/>
+      <c r="C42" s="30"/>
+      <c r="D42" s="30"/>
     </row>
     <row r="43" spans="1:4">
-      <c r="A43" s="31"/>
-      <c r="B43" s="31"/>
-      <c r="C43" s="31"/>
-      <c r="D43" s="31"/>
+      <c r="A43" s="30"/>
+      <c r="B43" s="30"/>
+      <c r="C43" s="30"/>
+      <c r="D43" s="30"/>
     </row>
     <row r="44" spans="1:4">
-      <c r="A44" s="31"/>
-      <c r="B44" s="31"/>
-      <c r="C44" s="31"/>
-      <c r="D44" s="31"/>
+      <c r="A44" s="30"/>
+      <c r="B44" s="30"/>
+      <c r="C44" s="30"/>
+      <c r="D44" s="30"/>
     </row>
     <row r="45" spans="1:4">
-      <c r="A45" s="31"/>
-      <c r="B45" s="31"/>
-      <c r="C45" s="31"/>
-      <c r="D45" s="31"/>
+      <c r="A45" s="30"/>
+      <c r="B45" s="30"/>
+      <c r="C45" s="30"/>
+      <c r="D45" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2117,7 +2182,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D073E50-F226-4B6A-BC2C-397D6C68AFA7}">
   <sheetPr codeName="Tabelle5"/>
-  <dimension ref="A1:V36"/>
+  <dimension ref="A1:X36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="22.3984375" bestFit="1" customWidth="1"/>
@@ -2136,14 +2201,16 @@
     <col min="15" max="15" width="14.5" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="27.3984375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="20.19921875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="24.796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.5" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="22.19921875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="23.796875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="27.3984375" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="18.8984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.8984375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="1" customFormat="1">
+    <row r="1" spans="1:24" s="1" customFormat="1">
       <c r="A1" s="5" t="s">
         <v>204</v>
       </c>
@@ -2210,8 +2277,14 @@
       <c r="V1" s="5" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="2" spans="1:22">
+      <c r="W1" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="X1" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2274,8 +2347,14 @@
       <c r="V2" s="2" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="3" spans="1:22">
+      <c r="W2" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -2342,8 +2421,14 @@
       <c r="V3" s="2" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="4" spans="1:22">
+      <c r="W3" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -2398,8 +2483,17 @@
       <c r="U4" s="2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="5" spans="1:22">
+      <c r="V4" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="W4" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -2436,8 +2530,14 @@
       <c r="U5" s="2" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="6" spans="1:22">
+      <c r="W5" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="X5" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -2474,8 +2574,14 @@
       <c r="U6" s="2" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="7" spans="1:22">
+      <c r="W6" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24">
       <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
@@ -2501,13 +2607,19 @@
         <v>199</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>99</v>
+        <v>260</v>
       </c>
       <c r="U7" s="2" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="8" spans="1:22">
+      <c r="W7" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="X7" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -2533,13 +2645,19 @@
         <v>93</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="U8" s="2" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="9" spans="1:22">
+      <c r="W8" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -2554,13 +2672,19 @@
         <v>119</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>233</v>
+        <v>100</v>
       </c>
       <c r="U9" s="2" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="10" spans="1:22">
+      <c r="W9" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="X9" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
@@ -2576,13 +2700,19 @@
       </c>
       <c r="K10" s="15"/>
       <c r="R10" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="U10" s="2" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="11" spans="1:22">
+      <c r="W10" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="X10" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -2598,13 +2728,19 @@
       </c>
       <c r="K11" s="15"/>
       <c r="R11" s="2" t="s">
-        <v>86</v>
+        <v>234</v>
       </c>
       <c r="U11" s="2" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="12" spans="1:22">
+      <c r="W11" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="X11" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -2616,11 +2752,17 @@
       </c>
       <c r="E12" s="1"/>
       <c r="K12" s="15"/>
+      <c r="R12" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="U12" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="13" spans="1:22">
+      <c r="W12" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -2632,8 +2774,14 @@
       </c>
       <c r="E13" s="1"/>
       <c r="K13" s="15"/>
-    </row>
-    <row r="14" spans="1:22">
+      <c r="R13" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="W13" s="3" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -2645,8 +2793,11 @@
       </c>
       <c r="E14" s="1"/>
       <c r="K14" s="15"/>
-    </row>
-    <row r="15" spans="1:22">
+      <c r="W14" s="3" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -2658,8 +2809,11 @@
       </c>
       <c r="E15" s="1"/>
       <c r="K15" s="15"/>
-    </row>
-    <row r="16" spans="1:22">
+      <c r="W15" s="3" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -2671,8 +2825,11 @@
       </c>
       <c r="E16" s="1"/>
       <c r="K16" s="15"/>
-    </row>
-    <row r="17" spans="1:11">
+      <c r="W16" s="3" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -2684,8 +2841,11 @@
       </c>
       <c r="E17" s="1"/>
       <c r="K17" s="15"/>
-    </row>
-    <row r="18" spans="1:11">
+      <c r="W17" s="3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
@@ -2697,8 +2857,11 @@
       </c>
       <c r="E18" s="1"/>
       <c r="K18" s="15"/>
-    </row>
-    <row r="19" spans="1:11">
+      <c r="W18" s="3" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -2710,8 +2873,11 @@
       </c>
       <c r="E19" s="1"/>
       <c r="K19" s="15"/>
-    </row>
-    <row r="20" spans="1:11">
+      <c r="W19" s="3" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
@@ -2723,8 +2889,11 @@
       </c>
       <c r="E20" s="1"/>
       <c r="K20" s="15"/>
-    </row>
-    <row r="21" spans="1:11">
+      <c r="W20" s="3" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -2736,8 +2905,11 @@
       </c>
       <c r="E21" s="1"/>
       <c r="K21" s="15"/>
-    </row>
-    <row r="22" spans="1:11">
+      <c r="W21" s="3" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
@@ -2746,7 +2918,7 @@
       </c>
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:23">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
@@ -2755,55 +2927,55 @@
       </c>
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:23">
       <c r="B24" s="2" t="s">
         <v>44</v>
       </c>
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:23">
       <c r="B25" s="2" t="s">
         <v>45</v>
       </c>
       <c r="E25" s="1"/>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:23">
       <c r="B26" s="2" t="s">
         <v>46</v>
       </c>
       <c r="E26" s="1"/>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:23">
       <c r="B27" s="2" t="s">
         <v>47</v>
       </c>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="1:11">
+    <row r="28" spans="1:23">
       <c r="B28" s="2" t="s">
         <v>48</v>
       </c>
       <c r="E28" s="1"/>
     </row>
-    <row r="29" spans="1:11">
+    <row r="29" spans="1:23">
       <c r="B29" s="2" t="s">
         <v>49</v>
       </c>
       <c r="E29" s="1"/>
     </row>
-    <row r="30" spans="1:11">
+    <row r="30" spans="1:23">
       <c r="B30" s="2" t="s">
         <v>50</v>
       </c>
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="1:11">
+    <row r="31" spans="1:23">
       <c r="B31" s="2" t="s">
         <v>51</v>
       </c>
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="1:11">
+    <row r="32" spans="1:23">
       <c r="B32" s="2" t="s">
         <v>52</v>
       </c>
@@ -2829,10 +3001,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="52lhtQEAIa0G0egiBOMSvDzW9IIazrxMJIqu++Msm7VrZR78YEHxwq0uV1phFxG1RVTLRGRFk7mWFXVjKblJ3g==" saltValue="LA2YV2MKD5bQ9zf69KBg+A==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V36">
-    <sortCondition sortBy="icon" ref="R9:R36"/>
-  </sortState>
+  <sheetProtection algorithmName="SHA-512" hashValue="ilEvpGmLo6a2O3ZAU+i9yQGGscrus6aYietO82VMOaIJdasi+nuCz4K4VGwvF5eoMx2reLQ9A/c/BCnrtsR9rw==" saltValue="4P2QQwj56WNptjDpbIU8kA==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Adapt dataset schemata and export function to change of organization and data source, fix typo at lhm_extern in mobidam schema
</commit_message>
<xml_diff>
--- a/ckanext/lhm/schemas/template_gdp.xlsx
+++ b/ckanext/lhm/schemas/template_gdp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\home\mb\p2\ckanext-lhm\ckanext\lhm\schemas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\home\mb\dev\ckanext-lhm\ckanext\lhm\schemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6607627-373A-4A41-A595-EF3B4A64B030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A61C35E-308A-4E06-891B-5CC483AD98BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1056" yWindow="1452" windowWidth="21792" windowHeight="10788" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
+    <workbookView xWindow="576" yWindow="0" windowWidth="23016" windowHeight="12108" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadaten" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="Wertelisten" sheetId="16" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Metadaten!$A$1:$K$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Metadaten!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="264">
   <si>
     <t>nein</t>
   </si>
@@ -259,9 +259,6 @@
   </si>
   <si>
     <t>Wert 10</t>
-  </si>
-  <si>
-    <t>Organisation *</t>
   </si>
   <si>
     <t>Externe Datenurheber *</t>
@@ -851,7 +848,13 @@
     <t>Link</t>
   </si>
   <si>
-    <t>1.3.3.</t>
+    <t>Abteilung *</t>
+  </si>
+  <si>
+    <t>1.3.6.</t>
+  </si>
+  <si>
+    <t>Metadatenschema *</t>
   </si>
 </sst>
 </file>
@@ -1453,7 +1456,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{860E5F97-3212-47C5-A469-BCE2C1CB3CAC}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="48.5" style="14" customWidth="1"/>
@@ -1502,7 +1505,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="18" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="12"/>
@@ -1517,7 +1520,7 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="12"/>
@@ -1532,7 +1535,7 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="12"/>
@@ -1547,7 +1550,7 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="16" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B5" s="21"/>
       <c r="C5" s="23"/>
@@ -1562,7 +1565,7 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="16" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B6" s="21"/>
       <c r="C6" s="21"/>
@@ -1577,7 +1580,7 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="12"/>
@@ -1592,7 +1595,7 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="12"/>
@@ -1622,7 +1625,7 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="16" t="s">
-        <v>71</v>
+        <v>261</v>
       </c>
       <c r="B10" s="21"/>
       <c r="C10" s="12"/>
@@ -1637,7 +1640,7 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B11" s="21"/>
       <c r="C11" s="12"/>
@@ -1652,7 +1655,7 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B12" s="22"/>
       <c r="C12" s="12"/>
@@ -1667,7 +1670,7 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B13" s="21"/>
       <c r="C13" s="12"/>
@@ -1682,7 +1685,7 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B14" s="19"/>
       <c r="C14" s="12"/>
@@ -1697,7 +1700,7 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="11" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B15" s="19"/>
       <c r="C15" s="12"/>
@@ -1727,7 +1730,7 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" s="16" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B17" s="21"/>
       <c r="C17" s="12"/>
@@ -1742,7 +1745,7 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" s="16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B18" s="21"/>
       <c r="C18" s="12"/>
@@ -1757,21 +1760,21 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="16" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B19" s="21"/>
       <c r="K19" s="17"/>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="16" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B20" s="21"/>
       <c r="K20" s="17"/>
     </row>
     <row r="21" spans="1:12">
       <c r="A21" s="16" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B21" s="21"/>
       <c r="C21" s="12"/>
@@ -1786,7 +1789,7 @@
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B22" s="21"/>
       <c r="C22" s="21"/>
@@ -1801,7 +1804,7 @@
     </row>
     <row r="23" spans="1:12">
       <c r="A23" s="16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B23" s="21"/>
       <c r="C23" s="12"/>
@@ -1816,7 +1819,7 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="16" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B24" s="21"/>
       <c r="C24" s="12"/>
@@ -1831,7 +1834,7 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25" s="16" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B25" s="21"/>
       <c r="C25" s="12"/>
@@ -1846,7 +1849,7 @@
     </row>
     <row r="26" spans="1:12">
       <c r="A26" s="16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B26" s="21"/>
       <c r="C26" s="12"/>
@@ -1861,7 +1864,7 @@
     </row>
     <row r="27" spans="1:12">
       <c r="A27" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B27" s="19"/>
       <c r="C27" s="24"/>
@@ -1876,7 +1879,7 @@
     </row>
     <row r="28" spans="1:12">
       <c r="A28" s="31" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B28" s="19"/>
       <c r="C28" s="24"/>
@@ -1891,7 +1894,7 @@
     </row>
     <row r="29" spans="1:12">
       <c r="A29" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B29" s="25"/>
       <c r="C29" s="12"/>
@@ -1907,7 +1910,7 @@
     </row>
     <row r="30" spans="1:12">
       <c r="A30" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B30" s="26"/>
       <c r="C30" s="12"/>
@@ -1923,7 +1926,7 @@
     </row>
     <row r="31" spans="1:12">
       <c r="A31" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B31" s="26"/>
       <c r="C31" s="12"/>
@@ -1939,11 +1942,9 @@
     </row>
     <row r="32" spans="1:12">
       <c r="A32" s="14" t="s">
-        <v>202</v>
-      </c>
-      <c r="B32" s="26" t="s">
-        <v>262</v>
-      </c>
+        <v>263</v>
+      </c>
+      <c r="B32" s="26"/>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
       <c r="E32" s="12"/>
@@ -1955,78 +1956,96 @@
       <c r="K32" s="12"/>
       <c r="L32" s="12"/>
     </row>
-    <row r="34" spans="1:4">
-      <c r="A34" s="14" t="s">
+    <row r="33" spans="1:12">
+      <c r="A33" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="B33" s="26" t="s">
+        <v>262</v>
+      </c>
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="12"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="12"/>
+      <c r="K33" s="12"/>
+      <c r="L33" s="12"/>
+    </row>
+    <row r="35" spans="1:12">
+      <c r="A35" s="14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12">
+      <c r="A36" s="14" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
-      <c r="A35" s="14" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4">
-      <c r="A37" s="29" t="s">
-        <v>193</v>
-      </c>
-      <c r="B37" s="30"/>
-      <c r="C37" s="30"/>
-      <c r="D37" s="30"/>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" s="30"/>
+    <row r="38" spans="1:12">
+      <c r="A38" s="29" t="s">
+        <v>192</v>
+      </c>
       <c r="B38" s="30"/>
       <c r="C38" s="30"/>
       <c r="D38" s="30"/>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:12">
       <c r="A39" s="30"/>
       <c r="B39" s="30"/>
       <c r="C39" s="30"/>
       <c r="D39" s="30"/>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:12">
       <c r="A40" s="30"/>
       <c r="B40" s="30"/>
       <c r="C40" s="30"/>
       <c r="D40" s="30"/>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:12">
       <c r="A41" s="30"/>
       <c r="B41" s="30"/>
       <c r="C41" s="30"/>
       <c r="D41" s="30"/>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:12">
       <c r="A42" s="30"/>
       <c r="B42" s="30"/>
       <c r="C42" s="30"/>
       <c r="D42" s="30"/>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:12">
       <c r="A43" s="30"/>
       <c r="B43" s="30"/>
       <c r="C43" s="30"/>
       <c r="D43" s="30"/>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:12">
       <c r="A44" s="30"/>
       <c r="B44" s="30"/>
       <c r="C44" s="30"/>
       <c r="D44" s="30"/>
     </row>
-    <row r="45" spans="1:4">
+    <row r="45" spans="1:12">
       <c r="A45" s="30"/>
       <c r="B45" s="30"/>
       <c r="C45" s="30"/>
       <c r="D45" s="30"/>
     </row>
+    <row r="46" spans="1:12">
+      <c r="A46" s="30"/>
+      <c r="B46" s="30"/>
+      <c r="C46" s="30"/>
+      <c r="D46" s="30"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A37:D45"/>
+    <mergeCell ref="A38:D46"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
-  <dataValidations xWindow="1350" yWindow="369" count="32">
+  <dataValidations xWindow="1350" yWindow="369" count="33">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thema | NAME_DER_TABELLE." prompt="Der Titel beteht aus dem Thema (für Geodatenpool: ehemals Datenbestand) und dem Namen der Tabelle in der Datenbank." sqref="B2" xr:uid="{7CC76290-C397-4A0D-82F8-39029843BD91}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Klare und prägnante Beschreibung des Datensatzes, damit auch Laien den Inhalt verstehen und einschätzen können. Dazu können neben dem konkreten Inhalt z.B. die räumliche Abdeckung, Vollständigkeit, Urheberschaft und Aktualität gehören." sqref="B4" xr:uid="{F0D16E7B-F9FC-4508-96CB-4EA176A334B4}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Schlagworte sind i.d.R. Substantive zur inhaltlichen Beschreibung des Datensatzes. Es können mehrere Schlagworte vergeben werden." sqref="B5" xr:uid="{623C178E-EC83-43E9-958F-0440F931AA20}"/>
@@ -2057,8 +2076,9 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Angabe der Team-E-Mailadresse des Datenverantwortlichen" sqref="B12" xr:uid="{BE4AF42B-6330-4B78-96B6-38C329A34190}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Mit High Value Datasets sind Daten gemeint, die in unter die DVO-HVD fallen. HVD-Daten sind per Definition immer auch Open Data." sqref="B24" xr:uid="{AC7FDAAF-072D-4534-A3F9-2DE40D62DD74}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Zusätzliche Hinweise zur Nutzung können unter 'Hinweise' mit Stichwort und Erklärung eingefügt werden. Diese müssen auch für Laien verständlich sein. Hinweise können z.B. zu vertraglichen Bedingungen oder Besonderheiten des Datensatzes erfolgen." sqref="B27" xr:uid="{4DD816CA-8275-41A8-B3C6-1162E00F43EE}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Die Datenquelle bezeichnet das System aus dem die Daten bezogen werden können, bspw. Geodatenpool." sqref="B31" xr:uid="{4BB7D51D-AB96-4002-8175-8BC4894AA0F9}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Version des Formats dieser Excel-Vorlage" sqref="B32" xr:uid="{DE5565F3-E0DE-421D-8CEB-430905832D21}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Die Datenquelle bezeichnet das System aus dem die Daten bezogen werden können, z.B. Geodatenpool. An ihr hängen als CKAN owner_org außerdem die Bearbeitungsrechte des Metadatensatzes." sqref="B31" xr:uid="{4BB7D51D-AB96-4002-8175-8BC4894AA0F9}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Version des Formats dieser Excel-Vorlage" sqref="B33" xr:uid="{DE5565F3-E0DE-421D-8CEB-430905832D21}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Das Metadatenschema bezeichnet das Schema, in dem die Metadaten gespeichert werden." sqref="B32" xr:uid="{D70F36C4-1632-4D58-9CC9-03CC7D92E979}"/>
   </dataValidations>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.78740157480314965" bottom="0.78740157480314965" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="64" fitToWidth="0" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -2082,22 +2102,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="27" t="s">
+        <v>182</v>
+      </c>
+      <c r="B1" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="B1" s="27" t="s">
-        <v>184</v>
-      </c>
       <c r="C1" s="27" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D1" s="27" t="s">
         <v>57</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F1" s="27" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -2124,16 +2144,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="27" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C1" s="27" t="s">
         <v>61</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -2158,16 +2178,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="27" t="s">
+        <v>185</v>
+      </c>
+      <c r="C1" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="27" t="s">
-        <v>186</v>
-      </c>
-      <c r="C1" s="27" t="s">
-        <v>88</v>
-      </c>
       <c r="D1" s="27" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2212,76 +2232,76 @@
   <sheetData>
     <row r="1" spans="1:24" s="1" customFormat="1">
       <c r="A1" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="Q1" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="R1" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="O1" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="Q1" s="5" t="s">
+      <c r="S1" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="T1" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="U1" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="R1" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="S1" s="5" t="s">
+      <c r="V1" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="T1" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="U1" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="V1" s="5" t="s">
-        <v>228</v>
-      </c>
       <c r="W1" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="X1" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:24">
@@ -2292,66 +2312,66 @@
         <v>23</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K2" s="3"/>
       <c r="L2" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="N2" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="M2" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>163</v>
-      </c>
       <c r="O2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q2" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="P2" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="R2" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:24">
@@ -2362,70 +2382,70 @@
         <v>24</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O3" s="2" t="s">
         <v>0</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="X3" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:24">
@@ -2436,61 +2456,61 @@
         <v>25</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="W4" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="X4" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" spans="1:24">
@@ -2501,40 +2521,40 @@
         <v>26</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="U5" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="X5" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:24">
@@ -2545,40 +2565,40 @@
         <v>27</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="U6" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="W6" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:24">
@@ -2589,34 +2609,34 @@
         <v>28</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="N7" s="3" t="s">
         <v>17</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="U7" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="X7" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:24">
@@ -2627,34 +2647,34 @@
         <v>29</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="U8" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="W8" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="X8" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" spans="1:24">
@@ -2665,23 +2685,23 @@
         <v>30</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E9" s="1"/>
       <c r="G9" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="U9" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="W9" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="X9" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:24">
@@ -2692,24 +2712,24 @@
         <v>31</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E10" s="1"/>
       <c r="G10" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K10" s="15"/>
       <c r="R10" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="U10" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="W10" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="X10" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" spans="1:24">
@@ -2720,24 +2740,24 @@
         <v>32</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E11" s="1"/>
       <c r="G11" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K11" s="15"/>
       <c r="R11" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="W11" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="X11" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:24">
@@ -2748,18 +2768,18 @@
         <v>33</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E12" s="1"/>
       <c r="K12" s="15"/>
       <c r="R12" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="U12" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="W12" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="13" spans="1:24">
@@ -2770,15 +2790,15 @@
         <v>34</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E13" s="1"/>
       <c r="K13" s="15"/>
       <c r="R13" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="W13" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14" spans="1:24">
@@ -2789,12 +2809,12 @@
         <v>35</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E14" s="1"/>
       <c r="K14" s="15"/>
       <c r="W14" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15" spans="1:24">
@@ -2805,12 +2825,12 @@
         <v>36</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E15" s="1"/>
       <c r="K15" s="15"/>
       <c r="W15" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16" spans="1:24">
@@ -2821,12 +2841,12 @@
         <v>37</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E16" s="1"/>
       <c r="K16" s="15"/>
       <c r="W16" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="17" spans="1:23">
@@ -2837,12 +2857,12 @@
         <v>38</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E17" s="1"/>
       <c r="K17" s="15"/>
       <c r="W17" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="18" spans="1:23">
@@ -2853,12 +2873,12 @@
         <v>39</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E18" s="1"/>
       <c r="K18" s="15"/>
       <c r="W18" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:23">
@@ -2869,12 +2889,12 @@
         <v>40</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E19" s="1"/>
       <c r="K19" s="15"/>
       <c r="W19" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="20" spans="1:23">
@@ -2882,15 +2902,15 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E20" s="1"/>
       <c r="K20" s="15"/>
       <c r="W20" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="21" spans="1:23">
@@ -2901,12 +2921,12 @@
         <v>41</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E21" s="1"/>
       <c r="K21" s="15"/>
       <c r="W21" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="22" spans="1:23">

</xml_diff>

<commit_message>
Adapt export to rearangement organizations - groups
</commit_message>
<xml_diff>
--- a/ckanext/lhm/schemas/template_gdp.xlsx
+++ b/ckanext/lhm/schemas/template_gdp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\home\mb\dev\ckanext-lhm\ckanext\lhm\schemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A61C35E-308A-4E06-891B-5CC483AD98BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1761557-9049-4F8C-A29C-CFC3539A09A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="576" yWindow="0" windowWidth="23016" windowHeight="12108" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadaten" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="265">
   <si>
     <t>nein</t>
   </si>
@@ -749,12 +749,6 @@
     <t>LHM_MD_datenquelle</t>
   </si>
   <si>
-    <t>Geodatenpool</t>
-  </si>
-  <si>
-    <t>Mobidam</t>
-  </si>
-  <si>
     <t>Attribut</t>
   </si>
   <si>
@@ -855,6 +849,15 @@
   </si>
   <si>
     <t>Metadatenschema *</t>
+  </si>
+  <si>
+    <t>GeoDatenPool</t>
+  </si>
+  <si>
+    <t>MobidaM</t>
+  </si>
+  <si>
+    <t>LHM_MD_metadatenschema</t>
   </si>
 </sst>
 </file>
@@ -1625,7 +1628,7 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="16" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B10" s="21"/>
       <c r="C10" s="12"/>
@@ -1942,7 +1945,7 @@
     </row>
     <row r="32" spans="1:12">
       <c r="A32" s="14" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B32" s="26"/>
       <c r="C32" s="12"/>
@@ -1961,7 +1964,7 @@
         <v>201</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>
@@ -2147,13 +2150,13 @@
         <v>84</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C1" s="27" t="s">
         <v>61</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -2202,7 +2205,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D073E50-F226-4B6A-BC2C-397D6C68AFA7}">
   <sheetPr codeName="Tabelle5"/>
-  <dimension ref="A1:X36"/>
+  <dimension ref="A1:Y36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="22.3984375" bestFit="1" customWidth="1"/>
@@ -2228,9 +2231,10 @@
     <col min="22" max="22" width="18.8984375" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="16.8984375" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="21.796875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="24.296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1">
+    <row r="1" spans="1:25" s="1" customFormat="1">
       <c r="A1" s="5" t="s">
         <v>203</v>
       </c>
@@ -2298,13 +2302,16 @@
         <v>227</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="X1" s="5" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="2" spans="1:24">
+        <v>233</v>
+      </c>
+      <c r="Y1" s="5" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2365,16 +2372,19 @@
         <v>92</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>228</v>
+        <v>262</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="X2" s="2" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="3" spans="1:24">
+      <c r="Y2" s="2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -2439,16 +2449,19 @@
         <v>91</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>229</v>
+        <v>263</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="X3" s="2" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="4" spans="1:24">
+      <c r="Y3" s="2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -2504,16 +2517,19 @@
         <v>90</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="W4" s="3" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="X4" s="2" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="5" spans="1:24">
+      <c r="Y4" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -2551,13 +2567,13 @@
         <v>89</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="X5" s="2" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="6" spans="1:24">
+    <row r="6" spans="1:25">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -2595,13 +2611,13 @@
         <v>194</v>
       </c>
       <c r="W6" s="3" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="X6" s="2" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:25">
       <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
@@ -2627,19 +2643,19 @@
         <v>198</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="U7" s="2" t="s">
         <v>193</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="X7" s="2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:25">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -2671,13 +2687,13 @@
         <v>195</v>
       </c>
       <c r="W8" s="3" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="X8" s="2" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="9" spans="1:24">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -2698,13 +2714,13 @@
         <v>197</v>
       </c>
       <c r="W9" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="X9" s="2" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="10" spans="1:24">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
@@ -2720,19 +2736,19 @@
       </c>
       <c r="K10" s="15"/>
       <c r="R10" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="U10" s="2" t="s">
         <v>196</v>
       </c>
       <c r="W10" s="3" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="X10" s="2" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="11" spans="1:24">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -2748,19 +2764,19 @@
       </c>
       <c r="K11" s="15"/>
       <c r="R11" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="U11" s="2" t="s">
         <v>198</v>
       </c>
       <c r="W11" s="3" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="X11" s="2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="12" spans="1:24">
+    <row r="12" spans="1:25">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -2779,10 +2795,10 @@
         <v>199</v>
       </c>
       <c r="W12" s="3" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="13" spans="1:24">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -2795,13 +2811,13 @@
       <c r="E13" s="1"/>
       <c r="K13" s="15"/>
       <c r="R13" s="2" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="W13" s="3" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="14" spans="1:24">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -2814,10 +2830,10 @@
       <c r="E14" s="1"/>
       <c r="K14" s="15"/>
       <c r="W14" s="3" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="15" spans="1:24">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -2830,10 +2846,10 @@
       <c r="E15" s="1"/>
       <c r="K15" s="15"/>
       <c r="W15" s="3" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="16" spans="1:24">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -2846,7 +2862,7 @@
       <c r="E16" s="1"/>
       <c r="K16" s="15"/>
       <c r="W16" s="3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="17" spans="1:23">
@@ -2862,7 +2878,7 @@
       <c r="E17" s="1"/>
       <c r="K17" s="15"/>
       <c r="W17" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="18" spans="1:23">
@@ -2894,7 +2910,7 @@
       <c r="E19" s="1"/>
       <c r="K19" s="15"/>
       <c r="W19" s="3" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="20" spans="1:23">
@@ -2910,7 +2926,7 @@
       <c r="E20" s="1"/>
       <c r="K20" s="15"/>
       <c r="W20" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="21" spans="1:23">
@@ -2926,7 +2942,7 @@
       <c r="E21" s="1"/>
       <c r="K21" s="15"/>
       <c r="W21" s="3" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="22" spans="1:23">
@@ -3021,7 +3037,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="ilEvpGmLo6a2O3ZAU+i9yQGGscrus6aYietO82VMOaIJdasi+nuCz4K4VGwvF5eoMx2reLQ9A/c/BCnrtsR9rw==" saltValue="4P2QQwj56WNptjDpbIU8kA==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="KFe0QCuD87thpdz4ck4fKMGzw5Q53fIojp2KlnoFb1hbwe+Rkl3kkRpWu6YGCCD+TcLUYpZIHFUAvwG7q3nsPA==" saltValue="7iA+BZblGrXOgve/UNdGnw==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>